<commit_message>
Update publication inventories and remove unused case studies
</commit_message>
<xml_diff>
--- a/dev/publication/LCIs/lci-pass_cars.xlsx
+++ b/dev/publication/LCIs/lci-pass_cars.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10510"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10531"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/romain/GitHub/trails/dev/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/romain/GitHub/trails/dev/publication/LCIs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C631062A-CCA5-6A48-8C0C-403529B9A3A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{52E87E28-82FC-FC42-880E-089C6EEE71DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="12580" yWindow="1600" windowWidth="25820" windowHeight="18980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4680" yWindow="660" windowWidth="25820" windowHeight="18980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="passenger cars" sheetId="1" r:id="rId1"/>
@@ -34,57 +34,321 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="428" uniqueCount="137">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="433" uniqueCount="137">
   <si>
     <t>Database</t>
   </si>
   <si>
+    <t>lci-trails</t>
+  </si>
+  <si>
     <t>Activity</t>
   </si>
   <si>
+    <t>reference product</t>
+  </si>
+  <si>
     <t>location</t>
   </si>
   <si>
+    <t>unit</t>
+  </si>
+  <si>
+    <t>lifetime [km]</t>
+  </si>
+  <si>
+    <t>fuel consumption [l/100 km]</t>
+  </si>
+  <si>
+    <t>lifetime [year]</t>
+  </si>
+  <si>
+    <t>average age [year]</t>
+  </si>
+  <si>
+    <t>comment</t>
+  </si>
+  <si>
+    <t>Example activitiy to test the import function of trails.</t>
+  </si>
+  <si>
+    <t>Exchanges</t>
+  </si>
+  <si>
+    <t>name</t>
+  </si>
+  <si>
+    <t>amount</t>
+  </si>
+  <si>
+    <t>categories</t>
+  </si>
+  <si>
+    <t>type</t>
+  </si>
+  <si>
+    <t>temporal_distribution</t>
+  </si>
+  <si>
+    <t>temporal_loc</t>
+  </si>
+  <si>
+    <t>temporal_scale</t>
+  </si>
+  <si>
+    <t>temporal_min</t>
+  </si>
+  <si>
+    <t>temporal_max</t>
+  </si>
+  <si>
+    <t>temporal_amount_source</t>
+  </si>
+  <si>
+    <t>transport, passenger, car, diesel</t>
+  </si>
+  <si>
+    <t>RER</t>
+  </si>
+  <si>
+    <t>kilometer</t>
+  </si>
+  <si>
+    <t>production</t>
+  </si>
+  <si>
+    <t>transport, passenger, car</t>
+  </si>
+  <si>
+    <t>market for brake wear emissions, passenger car</t>
+  </si>
+  <si>
     <t>GLO</t>
   </si>
   <si>
-    <t>reference product</t>
-  </si>
-  <si>
-    <t>type</t>
-  </si>
-  <si>
-    <t>unit</t>
-  </si>
-  <si>
-    <t>comment</t>
-  </si>
-  <si>
-    <t>Exchanges</t>
-  </si>
-  <si>
-    <t>name</t>
-  </si>
-  <si>
-    <t>amount</t>
-  </si>
-  <si>
-    <t>categories</t>
-  </si>
-  <si>
-    <t>production</t>
-  </si>
-  <si>
     <t>kilogram</t>
   </si>
   <si>
     <t>technosphere</t>
   </si>
   <si>
+    <t>brake wear emissions, passenger car</t>
+  </si>
+  <si>
+    <t>Occurs uniformly over the vehicle's use phase.</t>
+  </si>
+  <si>
+    <t>market for road wear emissions, passenger car</t>
+  </si>
+  <si>
+    <t>road wear emissions, passenger car</t>
+  </si>
+  <si>
+    <t>market for tyre wear emissions, passenger car</t>
+  </si>
+  <si>
+    <t>tyre wear emissions, passenger car</t>
+  </si>
+  <si>
+    <t>road construction</t>
+  </si>
+  <si>
     <t>RoW</t>
   </si>
   <si>
-    <t>RER</t>
+    <t>meter-year</t>
+  </si>
+  <si>
+    <t>road</t>
+  </si>
+  <si>
+    <t>The road has been continuously built between 40 years ago and last year.</t>
+  </si>
+  <si>
+    <t>maintenance, passenger car</t>
+  </si>
+  <si>
+    <t>passenger car maintenance</t>
+  </si>
+  <si>
+    <t>The car is being continuously maintained over the use phase.</t>
+  </si>
+  <si>
+    <t>market for road maintenance</t>
+  </si>
+  <si>
+    <t>road maintenance</t>
+  </si>
+  <si>
+    <t>The road undergoes maintenance uniformaly over the use phase.</t>
+  </si>
+  <si>
+    <t>diesel production, low-sulfur, petroleum refinery operation</t>
+  </si>
+  <si>
+    <t>Europe without Switzerland</t>
+  </si>
+  <si>
+    <t>diesel, low-sulfur</t>
+  </si>
+  <si>
+    <t>matrix</t>
+  </si>
+  <si>
+    <t>Here, the matrix-stored value is used, instead of porting the value and distirbuting it over years. Also, we indicate year-specific values. When absent, values under "amount" apply.</t>
+  </si>
+  <si>
+    <t>esterification of rape oil</t>
+  </si>
+  <si>
+    <t>fatty acid methyl ester</t>
+  </si>
+  <si>
+    <t>Carbon dioxide, fossil</t>
+  </si>
+  <si>
+    <t>air::urban air close to ground</t>
+  </si>
+  <si>
+    <t>biosphere</t>
+  </si>
+  <si>
+    <t>Carbon dioxide, non-fossil</t>
+  </si>
+  <si>
+    <t>passenger car production, diesel</t>
+  </si>
+  <si>
+    <t>passenger car, diesel</t>
+  </si>
+  <si>
+    <t>temporal_distribution: 2 = lognormal, 3 = normal, 4 = uniform and 5 = triangular.</t>
+  </si>
+  <si>
+    <t>Ethane</t>
+  </si>
+  <si>
+    <t>NMVOC, non-methane volatile organic compounds</t>
+  </si>
+  <si>
+    <t>Nickel II</t>
+  </si>
+  <si>
+    <t>Toluene</t>
+  </si>
+  <si>
+    <t>Styrene</t>
+  </si>
+  <si>
+    <t>Chromium III</t>
+  </si>
+  <si>
+    <t>Carbon monoxide, fossil</t>
+  </si>
+  <si>
+    <t>Copper ion</t>
+  </si>
+  <si>
+    <t>Sulfur dioxide</t>
+  </si>
+  <si>
+    <t>Ammonia</t>
+  </si>
+  <si>
+    <t>Lead II</t>
+  </si>
+  <si>
+    <t>Ethylene oxide</t>
+  </si>
+  <si>
+    <t>Benzaldehyde</t>
+  </si>
+  <si>
+    <t>Methane, fossil</t>
+  </si>
+  <si>
+    <t>Selenium IV</t>
+  </si>
+  <si>
+    <t>PAH, polycyclic aromatic hydrocarbons</t>
+  </si>
+  <si>
+    <t>Benzene</t>
+  </si>
+  <si>
+    <t>Pentane</t>
+  </si>
+  <si>
+    <t>Acrolein</t>
+  </si>
+  <si>
+    <t>Heptane</t>
+  </si>
+  <si>
+    <t>Formaldehyde</t>
+  </si>
+  <si>
+    <t>Cadmium II</t>
+  </si>
+  <si>
+    <t>Dinitrogen monoxide</t>
+  </si>
+  <si>
+    <t>Methyl ethyl ketone</t>
+  </si>
+  <si>
+    <t>Hydrocarbons, aliphatic, alkanes, cyclic</t>
+  </si>
+  <si>
+    <t>Chromium VI</t>
+  </si>
+  <si>
+    <t>Propane</t>
+  </si>
+  <si>
+    <t>o-Xylene</t>
+  </si>
+  <si>
+    <t>Acetaldehyde</t>
+  </si>
+  <si>
+    <t>Nitrogen oxides</t>
+  </si>
+  <si>
+    <t>Mercury II</t>
+  </si>
+  <si>
+    <t>Propylene oxide</t>
+  </si>
+  <si>
+    <t>Acetone</t>
+  </si>
+  <si>
+    <t>Particulate Matter, &lt; 2.5 um</t>
+  </si>
+  <si>
+    <t>Zinc II</t>
+  </si>
+  <si>
+    <t>Butane</t>
+  </si>
+  <si>
+    <t>m-Xylene</t>
+  </si>
+  <si>
+    <t>electricity consumption [kWh/100 km]</t>
+  </si>
+  <si>
+    <t>transport, passenger, car, battery electric</t>
+  </si>
+  <si>
+    <t>market for used Li-ion battery</t>
+  </si>
+  <si>
+    <t>used Li-ion battery</t>
+  </si>
+  <si>
+    <t>maintenance, passenger car, electric, without battery</t>
   </si>
   <si>
     <t>market group for electricity, low voltage</t>
@@ -96,300 +360,57 @@
     <t>electricity, low voltage</t>
   </si>
   <si>
-    <t>kilometer</t>
-  </si>
-  <si>
-    <t>biosphere</t>
-  </si>
-  <si>
-    <t>air::urban air close to ground</t>
-  </si>
-  <si>
-    <t>Acetaldehyde</t>
-  </si>
-  <si>
-    <t>Acetone</t>
-  </si>
-  <si>
-    <t>Acrolein</t>
-  </si>
-  <si>
-    <t>Ammonia</t>
-  </si>
-  <si>
-    <t>Benzaldehyde</t>
-  </si>
-  <si>
-    <t>Benzene</t>
-  </si>
-  <si>
-    <t>Butane</t>
-  </si>
-  <si>
-    <t>Carbon dioxide, fossil</t>
-  </si>
-  <si>
-    <t>Carbon monoxide, fossil</t>
-  </si>
-  <si>
-    <t>Chromium VI</t>
-  </si>
-  <si>
-    <t>Dinitrogen monoxide</t>
-  </si>
-  <si>
-    <t>Ethane</t>
-  </si>
-  <si>
-    <t>Formaldehyde</t>
-  </si>
-  <si>
-    <t>Heptane</t>
-  </si>
-  <si>
-    <t>Methane, fossil</t>
-  </si>
-  <si>
-    <t>Methyl ethyl ketone</t>
-  </si>
-  <si>
-    <t>Nitrogen oxides</t>
-  </si>
-  <si>
-    <t>PAH, polycyclic aromatic hydrocarbons</t>
-  </si>
-  <si>
-    <t>Pentane</t>
-  </si>
-  <si>
-    <t>Propane</t>
-  </si>
-  <si>
-    <t>Styrene</t>
-  </si>
-  <si>
-    <t>Sulfur dioxide</t>
-  </si>
-  <si>
-    <t>Toluene</t>
-  </si>
-  <si>
-    <t>m-Xylene</t>
-  </si>
-  <si>
-    <t>maintenance, passenger car</t>
-  </si>
-  <si>
-    <t>passenger car maintenance</t>
-  </si>
-  <si>
-    <t>market for brake wear emissions, passenger car</t>
-  </si>
-  <si>
-    <t>brake wear emissions, passenger car</t>
-  </si>
-  <si>
-    <t>meter-year</t>
-  </si>
-  <si>
-    <t>road</t>
-  </si>
-  <si>
-    <t>market for road maintenance</t>
-  </si>
-  <si>
-    <t>road maintenance</t>
-  </si>
-  <si>
-    <t>market for road wear emissions, passenger car</t>
-  </si>
-  <si>
-    <t>road wear emissions, passenger car</t>
-  </si>
-  <si>
-    <t>market for tyre wear emissions, passenger car</t>
-  </si>
-  <si>
-    <t>tyre wear emissions, passenger car</t>
-  </si>
-  <si>
-    <t>o-Xylene</t>
-  </si>
-  <si>
-    <t>diesel, low-sulfur</t>
-  </si>
-  <si>
-    <t>NMVOC, non-methane volatile organic compounds</t>
-  </si>
-  <si>
-    <t>Nickel II</t>
-  </si>
-  <si>
-    <t>Chromium III</t>
-  </si>
-  <si>
-    <t>Copper ion</t>
-  </si>
-  <si>
-    <t>Lead II</t>
-  </si>
-  <si>
-    <t>Ethylene oxide</t>
-  </si>
-  <si>
-    <t>Selenium IV</t>
-  </si>
-  <si>
-    <t>Cadmium II</t>
-  </si>
-  <si>
-    <t>Hydrocarbons, aliphatic, alkanes, cyclic</t>
-  </si>
-  <si>
-    <t>Mercury II</t>
-  </si>
-  <si>
-    <t>Propylene oxide</t>
-  </si>
-  <si>
-    <t>Particulate Matter, &lt; 2.5 um</t>
-  </si>
-  <si>
-    <t>Zinc II</t>
-  </si>
-  <si>
-    <t>passenger car, diesel</t>
-  </si>
-  <si>
-    <t>market for used Li-ion battery</t>
-  </si>
-  <si>
-    <t>used Li-ion battery</t>
-  </si>
-  <si>
-    <t>market for maintenance, passenger car, electric, without battery</t>
-  </si>
-  <si>
-    <t>maintenance, passenger car, electric, without battery</t>
+    <t>passenger car production, electric, without battery</t>
   </si>
   <si>
     <t>passenger car, electric, without battery</t>
   </si>
   <si>
-    <t>market for battery, Li-ion, LiMn2O4, rechargeable</t>
-  </si>
-  <si>
-    <t>battery, Li-ion, LiMn2O4, rechargeable</t>
-  </si>
-  <si>
-    <t>transport, passenger, car, diesel</t>
-  </si>
-  <si>
-    <t>transport, passenger, car, battery electric</t>
-  </si>
-  <si>
-    <t>transport, passenger, car</t>
-  </si>
-  <si>
-    <t>temporal_distribution</t>
-  </si>
-  <si>
-    <t>temporal_loc</t>
-  </si>
-  <si>
-    <t>temporal_scale</t>
-  </si>
-  <si>
-    <t>temporal_min</t>
-  </si>
-  <si>
-    <t>temporal_max</t>
-  </si>
-  <si>
-    <t>temporal_amount_source</t>
-  </si>
-  <si>
-    <t>lifetime [km]</t>
-  </si>
-  <si>
-    <t>lifetime [year]</t>
-  </si>
-  <si>
-    <t>average age [year]</t>
-  </si>
-  <si>
-    <t>passenger car production, diesel</t>
-  </si>
-  <si>
-    <t>passenger car production, electric, without battery</t>
-  </si>
-  <si>
-    <t>road construction</t>
-  </si>
-  <si>
-    <t>Occurs uniformly over the vehicle's use phase.</t>
-  </si>
-  <si>
-    <t>The road has been continuously built between 40 years ago and last year.</t>
-  </si>
-  <si>
-    <t>The car is being continuously maintained over the use phase.</t>
-  </si>
-  <si>
-    <t>The road undergoes maintenance uniformaly over the use phase.</t>
-  </si>
-  <si>
-    <t>lci-trails</t>
-  </si>
-  <si>
-    <t>Example activitiy to test the import function of trails.</t>
-  </si>
-  <si>
-    <t>Carbon dioxide, non-fossil</t>
-  </si>
-  <si>
-    <t>diesel production, low-sulfur, petroleum refinery operation</t>
-  </si>
-  <si>
-    <t>Europe without Switzerland</t>
-  </si>
-  <si>
-    <t>esterification of rape oil</t>
-  </si>
-  <si>
-    <t>fatty acid methyl ester</t>
-  </si>
-  <si>
-    <t>matrix</t>
-  </si>
-  <si>
-    <t>Here, the matrix-stored value is used, instead of porting the value and distirbuting it over years. Also, we indicate year-specific values. When absent, values under "amount" apply.</t>
-  </si>
-  <si>
-    <t>temporal_distribution: 2 = lognormal, 3 = normal, 4 = uniform and 5 = triangular.</t>
-  </si>
-  <si>
-    <t>fuel consumption [l/100 km]</t>
-  </si>
-  <si>
-    <t>electricity consumption [kWh/100 km]</t>
+    <t>battery production, Li-ion, LFP, rechargeable</t>
+  </si>
+  <si>
+    <t>CN</t>
+  </si>
+  <si>
+    <t>battery, Li-ion, LFP, rechargeable</t>
+  </si>
+  <si>
+    <t>heat</t>
+  </si>
+  <si>
+    <t>power [kW]</t>
+  </si>
+  <si>
+    <t>lifetime [y]</t>
+  </si>
+  <si>
+    <t>efficiency [.]</t>
+  </si>
+  <si>
+    <t>operation [hour/yer]</t>
+  </si>
+  <si>
+    <t>production [MJ/year]</t>
   </si>
   <si>
     <t>heating, from wood logs stove</t>
   </si>
   <si>
+    <t>megajoule</t>
+  </si>
+  <si>
+    <t>market for cleft timber, green, measured as dry mass</t>
+  </si>
+  <si>
+    <t>CH</t>
+  </si>
+  <si>
+    <t>cleft timber, green, measured as dry mass</t>
+  </si>
+  <si>
     <t>furnace production, logs, 30kW</t>
   </si>
   <si>
-    <t>market for cleft timber, green, measured as dry mass</t>
-  </si>
-  <si>
-    <t>cleft timber, green, measured as dry mass</t>
-  </si>
-  <si>
-    <t>CH</t>
-  </si>
-  <si>
     <t>furnace, logs, 30kW</t>
   </si>
   <si>
@@ -402,25 +423,10 @@
     <t>wood ash mixture, pure</t>
   </si>
   <si>
-    <t>lifetime [y]</t>
-  </si>
-  <si>
-    <t>efficiency [.]</t>
-  </si>
-  <si>
-    <t>operation [hour/yer]</t>
-  </si>
-  <si>
-    <t>production [MJ/year]</t>
-  </si>
-  <si>
-    <t>power [kW]</t>
-  </si>
-  <si>
-    <t>megajoule</t>
-  </si>
-  <si>
-    <t>heat</t>
+    <t>temporal_offsets</t>
+  </si>
+  <si>
+    <t>temporal_weights</t>
   </si>
   <si>
     <t>heating, from heat pump</t>
@@ -432,19 +438,13 @@
     <t>heat pump, 30kW</t>
   </si>
   <si>
+    <t>[-1,14]</t>
+  </si>
+  <si>
+    <t>[0.5,0.5]</t>
+  </si>
+  <si>
     <t>1,1,1,2-Tetrafluoroethane</t>
-  </si>
-  <si>
-    <t>temporal_offsets</t>
-  </si>
-  <si>
-    <t>temporal_weights</t>
-  </si>
-  <si>
-    <t>[0.5,0.5]</t>
-  </si>
-  <si>
-    <t>[-1,14]</t>
   </si>
 </sst>
 </file>
@@ -499,9 +499,9 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -509,6 +509,9 @@
     <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
@@ -812,11 +815,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:R84"/>
+  <dimension ref="A1:R85"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="49.83203125" customWidth="1"/>
-    <col min="2" max="2" width="30.1640625" customWidth="1"/>
+    <col min="2" max="2" width="15.1640625" customWidth="1"/>
     <col min="3" max="6" width="8.6640625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="11.5" customWidth="1"/>
     <col min="11" max="11" width="26.5" customWidth="1"/>
@@ -833,12 +836,12 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>101</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:18" s="1" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B3" s="1" t="str">
         <f>A14</f>
@@ -847,7 +850,7 @@
     </row>
     <row r="4" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B4" t="str">
         <f>K14</f>
@@ -856,7 +859,7 @@
     </row>
     <row r="5" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="B5" t="str">
         <f>G14</f>
@@ -865,7 +868,7 @@
     </row>
     <row r="6" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B6" t="str">
         <f>I14</f>
@@ -874,7 +877,7 @@
     </row>
     <row r="7" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>91</v>
+        <v>6</v>
       </c>
       <c r="B7">
         <v>150000</v>
@@ -882,7 +885,7 @@
     </row>
     <row r="8" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>111</v>
+        <v>7</v>
       </c>
       <c r="B8">
         <v>5</v>
@@ -890,7 +893,7 @@
     </row>
     <row r="9" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>92</v>
+        <v>8</v>
       </c>
       <c r="B9">
         <v>16</v>
@@ -898,7 +901,7 @@
     </row>
     <row r="10" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>93</v>
+        <v>9</v>
       </c>
       <c r="B10">
         <v>8</v>
@@ -906,23 +909,23 @@
     </row>
     <row r="11" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>102</v>
+        <v>11</v>
       </c>
     </row>
     <row r="12" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A12" s="1" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
     </row>
     <row r="13" spans="1:18" s="1" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A13" s="1" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="C13" s="1">
         <v>2020</v>
@@ -937,65 +940,66 @@
         <v>2080</v>
       </c>
       <c r="G13" s="1" t="s">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H13" s="1" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="I13" s="1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J13" s="1" t="s">
-        <v>5</v>
+        <v>16</v>
       </c>
       <c r="K13" s="1" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L13" s="1" t="s">
-        <v>85</v>
+        <v>17</v>
       </c>
       <c r="M13" s="1" t="s">
-        <v>86</v>
+        <v>18</v>
       </c>
       <c r="N13" s="1" t="s">
-        <v>87</v>
+        <v>19</v>
       </c>
       <c r="O13" s="1" t="s">
-        <v>88</v>
+        <v>20</v>
       </c>
       <c r="P13" s="1" t="s">
-        <v>89</v>
+        <v>21</v>
       </c>
       <c r="Q13" s="1" t="s">
-        <v>90</v>
+        <v>22</v>
       </c>
       <c r="R13" s="1" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
     </row>
     <row r="14" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>82</v>
+        <v>23</v>
       </c>
       <c r="B14">
-        <v>1</v>
+        <f>B7</f>
+        <v>150000</v>
       </c>
       <c r="G14" t="s">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="I14" t="s">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="J14" t="s">
-        <v>12</v>
+        <v>26</v>
       </c>
       <c r="K14" t="s">
-        <v>84</v>
+        <v>27</v>
       </c>
     </row>
     <row r="15" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>49</v>
+        <v>28</v>
       </c>
       <c r="B15" s="2">
         <v>-1.3998809999999999</v>
@@ -1005,16 +1009,16 @@
       <c r="E15" s="2"/>
       <c r="F15" s="2"/>
       <c r="G15" t="s">
-        <v>3</v>
+        <v>29</v>
       </c>
       <c r="I15" t="s">
-        <v>13</v>
+        <v>30</v>
       </c>
       <c r="J15" t="s">
-        <v>14</v>
+        <v>31</v>
       </c>
       <c r="K15" t="s">
-        <v>50</v>
+        <v>32</v>
       </c>
       <c r="L15">
         <v>4</v>
@@ -1031,12 +1035,12 @@
         <v>8</v>
       </c>
       <c r="R15" t="s">
-        <v>97</v>
+        <v>33</v>
       </c>
     </row>
     <row r="16" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>55</v>
+        <v>34</v>
       </c>
       <c r="B16" s="2">
         <v>-3.0797382</v>
@@ -1046,16 +1050,16 @@
       <c r="E16" s="2"/>
       <c r="F16" s="2"/>
       <c r="G16" t="s">
-        <v>3</v>
+        <v>29</v>
       </c>
       <c r="I16" t="s">
-        <v>13</v>
+        <v>30</v>
       </c>
       <c r="J16" t="s">
-        <v>14</v>
+        <v>31</v>
       </c>
       <c r="K16" t="s">
-        <v>56</v>
+        <v>35</v>
       </c>
       <c r="L16">
         <v>4</v>
@@ -1072,12 +1076,12 @@
         <v>8</v>
       </c>
       <c r="R16" t="s">
-        <v>97</v>
+        <v>33</v>
       </c>
     </row>
     <row r="17" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>57</v>
+        <v>36</v>
       </c>
       <c r="B17" s="2">
         <v>-18.009705</v>
@@ -1087,16 +1091,16 @@
       <c r="E17" s="2"/>
       <c r="F17" s="2"/>
       <c r="G17" t="s">
-        <v>3</v>
+        <v>29</v>
       </c>
       <c r="I17" t="s">
-        <v>13</v>
+        <v>30</v>
       </c>
       <c r="J17" t="s">
-        <v>14</v>
+        <v>31</v>
       </c>
       <c r="K17" t="s">
-        <v>58</v>
+        <v>37</v>
       </c>
       <c r="L17">
         <v>4</v>
@@ -1113,12 +1117,12 @@
         <v>8</v>
       </c>
       <c r="R17" t="s">
-        <v>97</v>
+        <v>33</v>
       </c>
     </row>
     <row r="18" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>96</v>
+        <v>38</v>
       </c>
       <c r="B18" s="2">
         <v>168.92946000000001</v>
@@ -1128,16 +1132,16 @@
       <c r="E18" s="2"/>
       <c r="F18" s="2"/>
       <c r="G18" t="s">
-        <v>15</v>
+        <v>39</v>
       </c>
       <c r="I18" t="s">
-        <v>51</v>
+        <v>40</v>
       </c>
       <c r="J18" t="s">
-        <v>14</v>
+        <v>31</v>
       </c>
       <c r="K18" t="s">
-        <v>52</v>
+        <v>41</v>
       </c>
       <c r="L18">
         <v>4</v>
@@ -1152,12 +1156,12 @@
         <v>-1</v>
       </c>
       <c r="R18" t="s">
-        <v>98</v>
+        <v>42</v>
       </c>
     </row>
     <row r="19" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="B19" s="2">
         <v>1.61290322580645</v>
@@ -1167,16 +1171,16 @@
       <c r="E19" s="2"/>
       <c r="F19" s="2"/>
       <c r="G19" t="s">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="I19" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J19" t="s">
-        <v>14</v>
+        <v>31</v>
       </c>
       <c r="K19" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="L19">
         <v>4</v>
@@ -1185,20 +1189,20 @@
         <v>0</v>
       </c>
       <c r="O19">
-        <f>$B$10-$B$9</f>
+        <f t="shared" ref="O19:O24" si="0">$B$10-$B$9</f>
         <v>-8</v>
       </c>
       <c r="P19">
-        <f>$B$9-$B$10</f>
+        <f t="shared" ref="P19:P24" si="1">$B$9-$B$10</f>
         <v>8</v>
       </c>
       <c r="R19" t="s">
-        <v>99</v>
+        <v>45</v>
       </c>
     </row>
     <row r="20" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>53</v>
+        <v>46</v>
       </c>
       <c r="B20" s="2">
         <v>39.799999999999997</v>
@@ -1208,16 +1212,16 @@
       <c r="E20" s="2"/>
       <c r="F20" s="2"/>
       <c r="G20" t="s">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="I20" t="s">
-        <v>51</v>
+        <v>40</v>
       </c>
       <c r="J20" t="s">
-        <v>14</v>
+        <v>31</v>
       </c>
       <c r="K20" t="s">
-        <v>54</v>
+        <v>47</v>
       </c>
       <c r="L20">
         <v>4</v>
@@ -1226,20 +1230,20 @@
         <v>0</v>
       </c>
       <c r="O20">
-        <f>$B$10-$B$9</f>
+        <f t="shared" si="0"/>
         <v>-8</v>
       </c>
       <c r="P20">
-        <f>$B$9-$B$10</f>
+        <f t="shared" si="1"/>
         <v>8</v>
       </c>
       <c r="R20" t="s">
-        <v>100</v>
+        <v>48</v>
       </c>
     </row>
     <row r="21" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>104</v>
+        <v>49</v>
       </c>
       <c r="B21" s="2">
         <f>B8*0.85/100*B7*1</f>
@@ -1262,16 +1266,16 @@
         <v>0</v>
       </c>
       <c r="G21" t="s">
-        <v>105</v>
+        <v>50</v>
       </c>
       <c r="I21" t="s">
-        <v>13</v>
+        <v>30</v>
       </c>
       <c r="J21" t="s">
-        <v>14</v>
+        <v>31</v>
       </c>
       <c r="K21" t="s">
-        <v>60</v>
+        <v>51</v>
       </c>
       <c r="L21">
         <v>4</v>
@@ -1280,23 +1284,23 @@
         <v>0</v>
       </c>
       <c r="O21">
-        <f>$B$10-$B$9</f>
+        <f t="shared" si="0"/>
         <v>-8</v>
       </c>
       <c r="P21">
-        <f>$B$9-$B$10</f>
+        <f t="shared" si="1"/>
         <v>8</v>
       </c>
       <c r="Q21" t="s">
-        <v>108</v>
+        <v>52</v>
       </c>
       <c r="R21" t="s">
-        <v>109</v>
+        <v>53</v>
       </c>
     </row>
     <row r="22" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>106</v>
+        <v>54</v>
       </c>
       <c r="B22" s="2">
         <f>B8*0.85/100*B7*0</f>
@@ -1319,16 +1323,16 @@
         <v>6375.0000000000009</v>
       </c>
       <c r="G22" t="s">
-        <v>105</v>
+        <v>50</v>
       </c>
       <c r="I22" t="s">
-        <v>13</v>
+        <v>30</v>
       </c>
       <c r="J22" t="s">
-        <v>14</v>
+        <v>31</v>
       </c>
       <c r="K22" t="s">
-        <v>107</v>
+        <v>55</v>
       </c>
       <c r="L22">
         <v>4</v>
@@ -1337,106 +1341,106 @@
         <v>0</v>
       </c>
       <c r="O22">
-        <f>$B$10-$B$9</f>
+        <f t="shared" si="0"/>
         <v>-8</v>
       </c>
       <c r="P22">
-        <f>$B$9-$B$10</f>
+        <f t="shared" si="1"/>
         <v>8</v>
       </c>
       <c r="Q22" t="s">
-        <v>108</v>
+        <v>52</v>
       </c>
       <c r="R22" t="s">
-        <v>109</v>
+        <v>53</v>
       </c>
     </row>
     <row r="23" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>30</v>
+        <v>56</v>
       </c>
       <c r="B23" s="3">
-        <f>B21*3.15</f>
+        <f t="shared" ref="B23:F24" si="2">B21*3.15</f>
         <v>20081.250000000004</v>
       </c>
       <c r="C23" s="3">
-        <f t="shared" ref="C23:F23" si="0">C21*3.15</f>
+        <f t="shared" si="2"/>
         <v>20081.250000000004</v>
       </c>
       <c r="D23" s="3">
+        <f t="shared" si="2"/>
+        <v>16065.000000000002</v>
+      </c>
+      <c r="E23" s="3">
+        <f t="shared" si="2"/>
+        <v>12048.750000000002</v>
+      </c>
+      <c r="F23" s="3">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="H23" t="s">
+        <v>57</v>
+      </c>
+      <c r="I23" t="s">
+        <v>30</v>
+      </c>
+      <c r="J23" t="s">
+        <v>58</v>
+      </c>
+      <c r="L23">
+        <v>4</v>
+      </c>
+      <c r="M23">
+        <v>0</v>
+      </c>
+      <c r="O23">
         <f t="shared" si="0"/>
-        <v>16065.000000000002</v>
-      </c>
-      <c r="E23" s="3">
-        <f t="shared" si="0"/>
-        <v>12048.750000000002</v>
-      </c>
-      <c r="F23" s="3">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="H23" t="s">
-        <v>22</v>
-      </c>
-      <c r="I23" t="s">
-        <v>13</v>
-      </c>
-      <c r="J23" t="s">
-        <v>21</v>
-      </c>
-      <c r="L23">
-        <v>4</v>
-      </c>
-      <c r="M23">
-        <v>0</v>
-      </c>
-      <c r="O23">
-        <f t="shared" ref="O23:O62" si="1">$B$10-$B$9</f>
         <v>-8</v>
       </c>
       <c r="P23">
-        <f t="shared" ref="P23:P62" si="2">$B$9-$B$10</f>
+        <f t="shared" si="1"/>
         <v>8</v>
       </c>
       <c r="Q23" t="s">
-        <v>108</v>
+        <v>52</v>
       </c>
       <c r="R23" t="s">
-        <v>109</v>
+        <v>53</v>
       </c>
     </row>
     <row r="24" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>103</v>
+        <v>59</v>
       </c>
       <c r="B24" s="3">
-        <f>B22*3.15</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="C24" s="3">
-        <f>C22*3.15</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="D24" s="3">
-        <f>D22*3.15</f>
+        <f t="shared" si="2"/>
         <v>4016.2500000000005</v>
       </c>
       <c r="E24" s="3">
-        <f>E22*3.15</f>
+        <f t="shared" si="2"/>
         <v>8032.5000000000009</v>
       </c>
       <c r="F24" s="3">
-        <f>F22*3.15</f>
+        <f t="shared" si="2"/>
         <v>20081.250000000004</v>
       </c>
       <c r="H24" t="s">
-        <v>22</v>
+        <v>57</v>
       </c>
       <c r="I24" t="s">
-        <v>13</v>
+        <v>30</v>
       </c>
       <c r="J24" t="s">
-        <v>21</v>
+        <v>58</v>
       </c>
       <c r="L24">
         <v>4</v>
@@ -1445,23 +1449,23 @@
         <v>0</v>
       </c>
       <c r="O24">
+        <f t="shared" si="0"/>
+        <v>-8</v>
+      </c>
+      <c r="P24">
         <f t="shared" si="1"/>
-        <v>-8</v>
-      </c>
-      <c r="P24">
-        <f t="shared" si="2"/>
         <v>8</v>
       </c>
       <c r="Q24" t="s">
-        <v>108</v>
+        <v>52</v>
       </c>
       <c r="R24" t="s">
-        <v>109</v>
+        <v>53</v>
       </c>
     </row>
     <row r="25" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>94</v>
+        <v>60</v>
       </c>
       <c r="B25" s="3">
         <v>2000</v>
@@ -1471,16 +1475,16 @@
       <c r="E25" s="2"/>
       <c r="F25" s="2"/>
       <c r="G25" t="s">
-        <v>3</v>
+        <v>29</v>
       </c>
       <c r="I25" t="s">
-        <v>13</v>
+        <v>30</v>
       </c>
       <c r="J25" t="s">
-        <v>14</v>
+        <v>31</v>
       </c>
       <c r="K25" t="s">
-        <v>74</v>
+        <v>61</v>
       </c>
       <c r="L25">
         <v>5</v>
@@ -1499,12 +1503,12 @@
         <v>-1</v>
       </c>
       <c r="R25" t="s">
-        <v>110</v>
+        <v>62</v>
       </c>
     </row>
     <row r="26" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>34</v>
+        <v>63</v>
       </c>
       <c r="B26" s="2">
         <v>1.6379999999999999E-2</v>
@@ -1514,13 +1518,13 @@
       <c r="E26" s="2"/>
       <c r="F26" s="2"/>
       <c r="H26" t="s">
-        <v>22</v>
+        <v>57</v>
       </c>
       <c r="I26" t="s">
-        <v>13</v>
+        <v>30</v>
       </c>
       <c r="J26" t="s">
-        <v>21</v>
+        <v>58</v>
       </c>
       <c r="L26">
         <v>4</v>
@@ -1529,33 +1533,33 @@
         <v>0</v>
       </c>
       <c r="O26">
-        <f t="shared" si="1"/>
+        <f t="shared" ref="O26:O62" si="3">$B$10-$B$9</f>
         <v>-8</v>
       </c>
       <c r="P26">
-        <f t="shared" si="2"/>
+        <f t="shared" ref="P26:P62" si="4">$B$9-$B$10</f>
         <v>8</v>
       </c>
     </row>
     <row r="27" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="B27" s="2">
-        <v>2.6310000000000002</v>
+        <v>2.6309999999999998</v>
       </c>
       <c r="C27" s="2"/>
       <c r="D27" s="2"/>
       <c r="E27" s="2"/>
       <c r="F27" s="2"/>
       <c r="H27" t="s">
-        <v>22</v>
+        <v>57</v>
       </c>
       <c r="I27" t="s">
-        <v>13</v>
+        <v>30</v>
       </c>
       <c r="J27" t="s">
-        <v>21</v>
+        <v>58</v>
       </c>
       <c r="L27">
         <v>4</v>
@@ -1564,17 +1568,17 @@
         <v>0</v>
       </c>
       <c r="O27">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>-8</v>
       </c>
       <c r="P27">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>8</v>
       </c>
     </row>
     <row r="28" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="B28" s="2">
         <v>7.3130358000000006E-4</v>
@@ -1584,13 +1588,13 @@
       <c r="E28" s="2"/>
       <c r="F28" s="2"/>
       <c r="H28" t="s">
-        <v>22</v>
+        <v>57</v>
       </c>
       <c r="I28" t="s">
-        <v>13</v>
+        <v>30</v>
       </c>
       <c r="J28" t="s">
-        <v>21</v>
+        <v>58</v>
       </c>
       <c r="L28">
         <v>4</v>
@@ -1599,17 +1603,17 @@
         <v>0</v>
       </c>
       <c r="O28">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>-8</v>
       </c>
       <c r="P28">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>8</v>
       </c>
     </row>
     <row r="29" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>45</v>
+        <v>66</v>
       </c>
       <c r="B29" s="2">
         <v>3.4229999999999997E-2</v>
@@ -1619,13 +1623,13 @@
       <c r="E29" s="2"/>
       <c r="F29" s="2"/>
       <c r="H29" t="s">
-        <v>22</v>
+        <v>57</v>
       </c>
       <c r="I29" t="s">
-        <v>13</v>
+        <v>30</v>
       </c>
       <c r="J29" t="s">
-        <v>21</v>
+        <v>58</v>
       </c>
       <c r="L29">
         <v>4</v>
@@ -1634,17 +1638,17 @@
         <v>0</v>
       </c>
       <c r="O29">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>-8</v>
       </c>
       <c r="P29">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>8</v>
       </c>
     </row>
     <row r="30" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
-        <v>43</v>
+        <v>67</v>
       </c>
       <c r="B30" s="2">
         <v>1.8360000000000001E-2</v>
@@ -1654,13 +1658,13 @@
       <c r="E30" s="2"/>
       <c r="F30" s="2"/>
       <c r="H30" t="s">
-        <v>22</v>
+        <v>57</v>
       </c>
       <c r="I30" t="s">
-        <v>13</v>
+        <v>30</v>
       </c>
       <c r="J30" t="s">
-        <v>21</v>
+        <v>58</v>
       </c>
       <c r="L30">
         <v>4</v>
@@ -1669,17 +1673,17 @@
         <v>0</v>
       </c>
       <c r="O30">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>-8</v>
       </c>
       <c r="P30">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>8</v>
       </c>
     </row>
     <row r="31" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="B31" s="2">
         <v>5.2235970000000004E-4</v>
@@ -1689,13 +1693,13 @@
       <c r="E31" s="2"/>
       <c r="F31" s="2"/>
       <c r="H31" t="s">
-        <v>22</v>
+        <v>57</v>
       </c>
       <c r="I31" t="s">
-        <v>13</v>
+        <v>30</v>
       </c>
       <c r="J31" t="s">
-        <v>21</v>
+        <v>58</v>
       </c>
       <c r="L31">
         <v>4</v>
@@ -1704,17 +1708,17 @@
         <v>0</v>
       </c>
       <c r="O31">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>-8</v>
       </c>
       <c r="P31">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>8</v>
       </c>
     </row>
     <row r="32" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
-        <v>31</v>
+        <v>69</v>
       </c>
       <c r="B32" s="2">
         <v>9.4649999999999999</v>
@@ -1724,13 +1728,13 @@
       <c r="E32" s="2"/>
       <c r="F32" s="2"/>
       <c r="H32" t="s">
-        <v>22</v>
+        <v>57</v>
       </c>
       <c r="I32" t="s">
-        <v>13</v>
+        <v>30</v>
       </c>
       <c r="J32" t="s">
-        <v>21</v>
+        <v>58</v>
       </c>
       <c r="L32">
         <v>4</v>
@@ -1739,17 +1743,17 @@
         <v>0</v>
       </c>
       <c r="O32">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>-8</v>
       </c>
       <c r="P32">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>8</v>
       </c>
     </row>
     <row r="33" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="B33" s="2">
         <v>1.7760229799999999E-2</v>
@@ -1759,13 +1763,13 @@
       <c r="E33" s="2"/>
       <c r="F33" s="2"/>
       <c r="H33" t="s">
-        <v>22</v>
+        <v>57</v>
       </c>
       <c r="I33" t="s">
-        <v>13</v>
+        <v>30</v>
       </c>
       <c r="J33" t="s">
-        <v>21</v>
+        <v>58</v>
       </c>
       <c r="L33">
         <v>4</v>
@@ -1774,17 +1778,17 @@
         <v>0</v>
       </c>
       <c r="O33">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>-8</v>
       </c>
       <c r="P33">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>8</v>
       </c>
     </row>
     <row r="34" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
-        <v>44</v>
+        <v>71</v>
       </c>
       <c r="B34" s="2">
         <v>0.20894388</v>
@@ -1794,13 +1798,13 @@
       <c r="E34" s="2"/>
       <c r="F34" s="2"/>
       <c r="H34" t="s">
-        <v>22</v>
+        <v>57</v>
       </c>
       <c r="I34" t="s">
-        <v>13</v>
+        <v>30</v>
       </c>
       <c r="J34" t="s">
-        <v>21</v>
+        <v>58</v>
       </c>
       <c r="L34">
         <v>4</v>
@@ -1809,17 +1813,17 @@
         <v>0</v>
       </c>
       <c r="O34">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>-8</v>
       </c>
       <c r="P34">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>8</v>
       </c>
     </row>
     <row r="35" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
-        <v>26</v>
+        <v>72</v>
       </c>
       <c r="B35" s="2">
         <v>0.167155104</v>
@@ -1829,13 +1833,13 @@
       <c r="E35" s="2"/>
       <c r="F35" s="2"/>
       <c r="H35" t="s">
-        <v>22</v>
+        <v>57</v>
       </c>
       <c r="I35" t="s">
-        <v>13</v>
+        <v>30</v>
       </c>
       <c r="J35" t="s">
-        <v>21</v>
+        <v>58</v>
       </c>
       <c r="L35">
         <v>4</v>
@@ -1844,17 +1848,17 @@
         <v>0</v>
       </c>
       <c r="O35">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>-8</v>
       </c>
       <c r="P35">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>8</v>
       </c>
     </row>
     <row r="36" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
-        <v>65</v>
+        <v>73</v>
       </c>
       <c r="B36" s="2">
         <v>8.6189350500000001E-10</v>
@@ -1864,13 +1868,13 @@
       <c r="E36" s="2"/>
       <c r="F36" s="2"/>
       <c r="H36" t="s">
-        <v>22</v>
+        <v>57</v>
       </c>
       <c r="I36" t="s">
-        <v>13</v>
+        <v>30</v>
       </c>
       <c r="J36" t="s">
-        <v>21</v>
+        <v>58</v>
       </c>
       <c r="L36">
         <v>4</v>
@@ -1879,17 +1883,17 @@
         <v>0</v>
       </c>
       <c r="O36">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>-8</v>
       </c>
       <c r="P36">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>8</v>
       </c>
     </row>
     <row r="37" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
-        <v>66</v>
+        <v>74</v>
       </c>
       <c r="B37" s="2">
         <v>0.54420000000000002</v>
@@ -1899,13 +1903,13 @@
       <c r="E37" s="2"/>
       <c r="F37" s="2"/>
       <c r="H37" t="s">
-        <v>22</v>
+        <v>57</v>
       </c>
       <c r="I37" t="s">
-        <v>13</v>
+        <v>30</v>
       </c>
       <c r="J37" t="s">
-        <v>21</v>
+        <v>58</v>
       </c>
       <c r="L37">
         <v>4</v>
@@ -1914,17 +1918,17 @@
         <v>0</v>
       </c>
       <c r="O37">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>-8</v>
       </c>
       <c r="P37">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>8</v>
       </c>
     </row>
     <row r="38" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
-        <v>27</v>
+        <v>75</v>
       </c>
       <c r="B38" s="2">
         <v>4.2674999999999998E-2</v>
@@ -1934,13 +1938,13 @@
       <c r="E38" s="2"/>
       <c r="F38" s="2"/>
       <c r="H38" t="s">
-        <v>22</v>
+        <v>57</v>
       </c>
       <c r="I38" t="s">
-        <v>13</v>
+        <v>30</v>
       </c>
       <c r="J38" t="s">
-        <v>21</v>
+        <v>58</v>
       </c>
       <c r="L38">
         <v>4</v>
@@ -1949,17 +1953,17 @@
         <v>0</v>
       </c>
       <c r="O38">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>-8</v>
       </c>
       <c r="P38">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>8</v>
       </c>
     </row>
     <row r="39" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
-        <v>37</v>
+        <v>76</v>
       </c>
       <c r="B39" s="2">
         <v>0.29849999999999999</v>
@@ -1969,13 +1973,13 @@
       <c r="E39" s="2"/>
       <c r="F39" s="2"/>
       <c r="H39" t="s">
-        <v>22</v>
+        <v>57</v>
       </c>
       <c r="I39" t="s">
-        <v>13</v>
+        <v>30</v>
       </c>
       <c r="J39" t="s">
-        <v>21</v>
+        <v>58</v>
       </c>
       <c r="L39">
         <v>4</v>
@@ -1984,33 +1988,33 @@
         <v>0</v>
       </c>
       <c r="O39">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>-8</v>
       </c>
       <c r="P39">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>8</v>
       </c>
     </row>
     <row r="40" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
-        <v>67</v>
+        <v>77</v>
       </c>
       <c r="B40" s="2">
-        <v>1.0447194000000001E-4</v>
+        <v>1.0447193999999999E-4</v>
       </c>
       <c r="C40" s="2"/>
       <c r="D40" s="2"/>
       <c r="E40" s="2"/>
       <c r="F40" s="2"/>
       <c r="H40" t="s">
-        <v>22</v>
+        <v>57</v>
       </c>
       <c r="I40" t="s">
-        <v>13</v>
+        <v>30</v>
       </c>
       <c r="J40" t="s">
-        <v>21</v>
+        <v>58</v>
       </c>
       <c r="L40">
         <v>4</v>
@@ -2019,17 +2023,17 @@
         <v>0</v>
       </c>
       <c r="O40">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>-8</v>
       </c>
       <c r="P40">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>8</v>
       </c>
     </row>
     <row r="41" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
-        <v>40</v>
+        <v>78</v>
       </c>
       <c r="B41" s="2">
         <v>1.9264625736000001E-3</v>
@@ -2039,13 +2043,13 @@
       <c r="E41" s="2"/>
       <c r="F41" s="2"/>
       <c r="H41" t="s">
-        <v>22</v>
+        <v>57</v>
       </c>
       <c r="I41" t="s">
-        <v>13</v>
+        <v>30</v>
       </c>
       <c r="J41" t="s">
-        <v>21</v>
+        <v>58</v>
       </c>
       <c r="L41">
         <v>4</v>
@@ -2054,17 +2058,17 @@
         <v>0</v>
       </c>
       <c r="O41">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>-8</v>
       </c>
       <c r="P41">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>8</v>
       </c>
     </row>
     <row r="42" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
-        <v>28</v>
+        <v>79</v>
       </c>
       <c r="B42" s="2">
         <v>9.8234999999999989E-2</v>
@@ -2074,13 +2078,13 @@
       <c r="E42" s="2"/>
       <c r="F42" s="2"/>
       <c r="H42" t="s">
-        <v>22</v>
+        <v>57</v>
       </c>
       <c r="I42" t="s">
-        <v>13</v>
+        <v>30</v>
       </c>
       <c r="J42" t="s">
-        <v>21</v>
+        <v>58</v>
       </c>
       <c r="L42">
         <v>4</v>
@@ -2089,17 +2093,17 @@
         <v>0</v>
       </c>
       <c r="O42">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>-8</v>
       </c>
       <c r="P42">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>8</v>
       </c>
     </row>
     <row r="43" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
-        <v>41</v>
+        <v>80</v>
       </c>
       <c r="B43" s="2">
         <v>1.9845000000000002E-3</v>
@@ -2109,13 +2113,13 @@
       <c r="E43" s="2"/>
       <c r="F43" s="2"/>
       <c r="H43" t="s">
-        <v>22</v>
+        <v>57</v>
       </c>
       <c r="I43" t="s">
-        <v>13</v>
+        <v>30</v>
       </c>
       <c r="J43" t="s">
-        <v>21</v>
+        <v>58</v>
       </c>
       <c r="L43">
         <v>4</v>
@@ -2124,17 +2128,17 @@
         <v>0</v>
       </c>
       <c r="O43">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>-8</v>
       </c>
       <c r="P43">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>8</v>
       </c>
     </row>
     <row r="44" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
-        <v>25</v>
+        <v>81</v>
       </c>
       <c r="B44" s="2">
         <v>0.17760000000000001</v>
@@ -2144,13 +2148,13 @@
       <c r="E44" s="2"/>
       <c r="F44" s="2"/>
       <c r="H44" t="s">
-        <v>22</v>
+        <v>57</v>
       </c>
       <c r="I44" t="s">
-        <v>13</v>
+        <v>30</v>
       </c>
       <c r="J44" t="s">
-        <v>21</v>
+        <v>58</v>
       </c>
       <c r="L44">
         <v>4</v>
@@ -2159,17 +2163,17 @@
         <v>0</v>
       </c>
       <c r="O44">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>-8</v>
       </c>
       <c r="P44">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>8</v>
       </c>
     </row>
     <row r="45" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
-        <v>36</v>
+        <v>82</v>
       </c>
       <c r="B45" s="2">
         <v>9.922499999999999E-3</v>
@@ -2179,13 +2183,13 @@
       <c r="E45" s="2"/>
       <c r="F45" s="2"/>
       <c r="H45" t="s">
-        <v>22</v>
+        <v>57</v>
       </c>
       <c r="I45" t="s">
-        <v>13</v>
+        <v>30</v>
       </c>
       <c r="J45" t="s">
-        <v>21</v>
+        <v>58</v>
       </c>
       <c r="L45">
         <v>4</v>
@@ -2194,17 +2198,17 @@
         <v>0</v>
       </c>
       <c r="O45">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>-8</v>
       </c>
       <c r="P45">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>8</v>
       </c>
     </row>
     <row r="46" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
-        <v>35</v>
+        <v>83</v>
       </c>
       <c r="B46" s="2">
         <v>0.59534999999999993</v>
@@ -2214,13 +2218,13 @@
       <c r="E46" s="2"/>
       <c r="F46" s="2"/>
       <c r="H46" t="s">
-        <v>22</v>
+        <v>57</v>
       </c>
       <c r="I46" t="s">
-        <v>13</v>
+        <v>30</v>
       </c>
       <c r="J46" t="s">
-        <v>21</v>
+        <v>58</v>
       </c>
       <c r="L46">
         <v>4</v>
@@ -2229,33 +2233,33 @@
         <v>0</v>
       </c>
       <c r="O46">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>-8</v>
       </c>
       <c r="P46">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>8</v>
       </c>
     </row>
     <row r="47" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
-        <v>68</v>
+        <v>84</v>
       </c>
       <c r="B47" s="2">
-        <v>1.0447194000000001E-4</v>
+        <v>1.0447193999999999E-4</v>
       </c>
       <c r="C47" s="2"/>
       <c r="D47" s="2"/>
       <c r="E47" s="2"/>
       <c r="F47" s="2"/>
       <c r="H47" t="s">
-        <v>22</v>
+        <v>57</v>
       </c>
       <c r="I47" t="s">
-        <v>13</v>
+        <v>30</v>
       </c>
       <c r="J47" t="s">
-        <v>21</v>
+        <v>58</v>
       </c>
       <c r="L47">
         <v>4</v>
@@ -2264,17 +2268,17 @@
         <v>0</v>
       </c>
       <c r="O47">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>-8</v>
       </c>
       <c r="P47">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>8</v>
       </c>
     </row>
     <row r="48" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
-        <v>33</v>
+        <v>85</v>
       </c>
       <c r="B48" s="2">
         <v>0.52235969999999998</v>
@@ -2284,13 +2288,13 @@
       <c r="E48" s="2"/>
       <c r="F48" s="2"/>
       <c r="H48" t="s">
-        <v>22</v>
+        <v>57</v>
       </c>
       <c r="I48" t="s">
-        <v>13</v>
+        <v>30</v>
       </c>
       <c r="J48" t="s">
-        <v>21</v>
+        <v>58</v>
       </c>
       <c r="L48">
         <v>4</v>
@@ -2299,33 +2303,33 @@
         <v>0</v>
       </c>
       <c r="O48">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>-8</v>
       </c>
       <c r="P48">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>8</v>
       </c>
     </row>
     <row r="49" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
-        <v>38</v>
+        <v>86</v>
       </c>
       <c r="B49" s="2">
-        <v>5.9535000000000005E-2</v>
+        <v>5.9534999999999998E-2</v>
       </c>
       <c r="C49" s="2"/>
       <c r="D49" s="2"/>
       <c r="E49" s="2"/>
       <c r="F49" s="2"/>
       <c r="H49" t="s">
-        <v>22</v>
+        <v>57</v>
       </c>
       <c r="I49" t="s">
-        <v>13</v>
+        <v>30</v>
       </c>
       <c r="J49" t="s">
-        <v>21</v>
+        <v>58</v>
       </c>
       <c r="L49">
         <v>4</v>
@@ -2334,17 +2338,17 @@
         <v>0</v>
       </c>
       <c r="O49">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>-8</v>
       </c>
       <c r="P49">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>8</v>
       </c>
     </row>
     <row r="50" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
-        <v>69</v>
+        <v>87</v>
       </c>
       <c r="B50" s="2">
         <v>3.2250000000000001E-2</v>
@@ -2354,13 +2358,13 @@
       <c r="E50" s="2"/>
       <c r="F50" s="2"/>
       <c r="H50" t="s">
-        <v>22</v>
+        <v>57</v>
       </c>
       <c r="I50" t="s">
-        <v>13</v>
+        <v>30</v>
       </c>
       <c r="J50" t="s">
-        <v>21</v>
+        <v>58</v>
       </c>
       <c r="L50">
         <v>4</v>
@@ -2369,17 +2373,17 @@
         <v>0</v>
       </c>
       <c r="O50">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>-8</v>
       </c>
       <c r="P50">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>8</v>
       </c>
     </row>
     <row r="51" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
-        <v>32</v>
+        <v>88</v>
       </c>
       <c r="B51" s="2">
         <v>1.0447194E-6</v>
@@ -2389,13 +2393,13 @@
       <c r="E51" s="2"/>
       <c r="F51" s="2"/>
       <c r="H51" t="s">
-        <v>22</v>
+        <v>57</v>
       </c>
       <c r="I51" t="s">
-        <v>13</v>
+        <v>30</v>
       </c>
       <c r="J51" t="s">
-        <v>21</v>
+        <v>58</v>
       </c>
       <c r="L51">
         <v>4</v>
@@ -2404,17 +2408,17 @@
         <v>0</v>
       </c>
       <c r="O51">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>-8</v>
       </c>
       <c r="P51">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>8</v>
       </c>
     </row>
     <row r="52" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
-        <v>42</v>
+        <v>89</v>
       </c>
       <c r="B52" s="2">
         <v>5.457E-3</v>
@@ -2424,13 +2428,13 @@
       <c r="E52" s="2"/>
       <c r="F52" s="2"/>
       <c r="H52" t="s">
-        <v>22</v>
+        <v>57</v>
       </c>
       <c r="I52" t="s">
-        <v>13</v>
+        <v>30</v>
       </c>
       <c r="J52" t="s">
-        <v>21</v>
+        <v>58</v>
       </c>
       <c r="L52">
         <v>4</v>
@@ -2439,33 +2443,33 @@
         <v>0</v>
       </c>
       <c r="O52">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>-8</v>
       </c>
       <c r="P52">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>8</v>
       </c>
     </row>
     <row r="53" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
-        <v>59</v>
+        <v>90</v>
       </c>
       <c r="B53" s="2">
-        <v>1.3396499999999999E-2</v>
+        <v>1.33965E-2</v>
       </c>
       <c r="C53" s="2"/>
       <c r="D53" s="2"/>
       <c r="E53" s="2"/>
       <c r="F53" s="2"/>
       <c r="H53" t="s">
-        <v>22</v>
+        <v>57</v>
       </c>
       <c r="I53" t="s">
-        <v>13</v>
+        <v>30</v>
       </c>
       <c r="J53" t="s">
-        <v>21</v>
+        <v>58</v>
       </c>
       <c r="L53">
         <v>4</v>
@@ -2474,33 +2478,33 @@
         <v>0</v>
       </c>
       <c r="O53">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>-8</v>
       </c>
       <c r="P53">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>8</v>
       </c>
     </row>
     <row r="54" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
-        <v>23</v>
+        <v>91</v>
       </c>
       <c r="B54" s="2">
-        <v>0.32099999999999995</v>
+        <v>0.32100000000000001</v>
       </c>
       <c r="C54" s="2"/>
       <c r="D54" s="2"/>
       <c r="E54" s="2"/>
       <c r="F54" s="2"/>
       <c r="H54" t="s">
-        <v>22</v>
+        <v>57</v>
       </c>
       <c r="I54" t="s">
-        <v>13</v>
+        <v>30</v>
       </c>
       <c r="J54" t="s">
-        <v>21</v>
+        <v>58</v>
       </c>
       <c r="L54">
         <v>4</v>
@@ -2509,17 +2513,17 @@
         <v>0</v>
       </c>
       <c r="O54">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>-8</v>
       </c>
       <c r="P54">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>8</v>
       </c>
     </row>
     <row r="55" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
-        <v>39</v>
+        <v>92</v>
       </c>
       <c r="B55" s="2">
         <v>101.589</v>
@@ -2529,13 +2533,13 @@
       <c r="E55" s="2"/>
       <c r="F55" s="2"/>
       <c r="H55" t="s">
-        <v>22</v>
+        <v>57</v>
       </c>
       <c r="I55" t="s">
-        <v>13</v>
+        <v>30</v>
       </c>
       <c r="J55" t="s">
-        <v>21</v>
+        <v>58</v>
       </c>
       <c r="L55">
         <v>4</v>
@@ -2544,17 +2548,17 @@
         <v>0</v>
       </c>
       <c r="O55">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>-8</v>
       </c>
       <c r="P55">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>8</v>
       </c>
     </row>
     <row r="56" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
-        <v>70</v>
+        <v>93</v>
       </c>
       <c r="B56" s="2">
         <v>2.0894388000000001E-7</v>
@@ -2564,13 +2568,13 @@
       <c r="E56" s="2"/>
       <c r="F56" s="2"/>
       <c r="H56" t="s">
-        <v>22</v>
+        <v>57</v>
       </c>
       <c r="I56" t="s">
-        <v>13</v>
+        <v>30</v>
       </c>
       <c r="J56" t="s">
-        <v>21</v>
+        <v>58</v>
       </c>
       <c r="L56">
         <v>4</v>
@@ -2579,33 +2583,33 @@
         <v>0</v>
       </c>
       <c r="O56">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>-8</v>
       </c>
       <c r="P56">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>8</v>
       </c>
     </row>
     <row r="57" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
-        <v>71</v>
+        <v>94</v>
       </c>
       <c r="B57" s="2">
-        <v>0.17864999999999998</v>
+        <v>0.17865</v>
       </c>
       <c r="C57" s="2"/>
       <c r="D57" s="2"/>
       <c r="E57" s="2"/>
       <c r="F57" s="2"/>
       <c r="H57" t="s">
-        <v>22</v>
+        <v>57</v>
       </c>
       <c r="I57" t="s">
-        <v>13</v>
+        <v>30</v>
       </c>
       <c r="J57" t="s">
-        <v>21</v>
+        <v>58</v>
       </c>
       <c r="L57">
         <v>4</v>
@@ -2614,17 +2618,17 @@
         <v>0</v>
       </c>
       <c r="O57">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>-8</v>
       </c>
       <c r="P57">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>8</v>
       </c>
     </row>
     <row r="58" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
-        <v>24</v>
+        <v>95</v>
       </c>
       <c r="B58" s="2">
         <v>0.14585999999999999</v>
@@ -2634,13 +2638,13 @@
       <c r="E58" s="2"/>
       <c r="F58" s="2"/>
       <c r="H58" t="s">
-        <v>22</v>
+        <v>57</v>
       </c>
       <c r="I58" t="s">
-        <v>13</v>
+        <v>30</v>
       </c>
       <c r="J58" t="s">
-        <v>21</v>
+        <v>58</v>
       </c>
       <c r="L58">
         <v>4</v>
@@ -2649,17 +2653,17 @@
         <v>0</v>
       </c>
       <c r="O58">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>-8</v>
       </c>
       <c r="P58">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>8</v>
       </c>
     </row>
     <row r="59" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
-        <v>72</v>
+        <v>96</v>
       </c>
       <c r="B59" s="2">
         <v>0.28719</v>
@@ -2669,13 +2673,13 @@
       <c r="E59" s="2"/>
       <c r="F59" s="2"/>
       <c r="H59" t="s">
-        <v>22</v>
+        <v>57</v>
       </c>
       <c r="I59" t="s">
-        <v>13</v>
+        <v>30</v>
       </c>
       <c r="J59" t="s">
-        <v>21</v>
+        <v>58</v>
       </c>
       <c r="L59">
         <v>4</v>
@@ -2684,17 +2688,17 @@
         <v>0</v>
       </c>
       <c r="O59">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>-8</v>
       </c>
       <c r="P59">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>8</v>
       </c>
     </row>
     <row r="60" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
-        <v>73</v>
+        <v>97</v>
       </c>
       <c r="B60" s="2">
         <v>1.0447194E-2</v>
@@ -2704,13 +2708,13 @@
       <c r="E60" s="2"/>
       <c r="F60" s="2"/>
       <c r="H60" t="s">
-        <v>22</v>
+        <v>57</v>
       </c>
       <c r="I60" t="s">
-        <v>13</v>
+        <v>30</v>
       </c>
       <c r="J60" t="s">
-        <v>21</v>
+        <v>58</v>
       </c>
       <c r="L60">
         <v>4</v>
@@ -2719,17 +2723,17 @@
         <v>0</v>
       </c>
       <c r="O60">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>-8</v>
       </c>
       <c r="P60">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>8</v>
       </c>
     </row>
     <row r="61" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
-        <v>29</v>
+        <v>98</v>
       </c>
       <c r="B61" s="2">
         <v>5.457E-3</v>
@@ -2739,13 +2743,13 @@
       <c r="E61" s="2"/>
       <c r="F61" s="2"/>
       <c r="H61" t="s">
-        <v>22</v>
+        <v>57</v>
       </c>
       <c r="I61" t="s">
-        <v>13</v>
+        <v>30</v>
       </c>
       <c r="J61" t="s">
-        <v>21</v>
+        <v>58</v>
       </c>
       <c r="L61">
         <v>4</v>
@@ -2754,17 +2758,17 @@
         <v>0</v>
       </c>
       <c r="O61">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>-8</v>
       </c>
       <c r="P61">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>8</v>
       </c>
     </row>
     <row r="62" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
-        <v>46</v>
+        <v>99</v>
       </c>
       <c r="B62" s="2">
         <v>3.0269999999999998E-2</v>
@@ -2774,13 +2778,13 @@
       <c r="E62" s="2"/>
       <c r="F62" s="2"/>
       <c r="H62" t="s">
-        <v>22</v>
+        <v>57</v>
       </c>
       <c r="I62" t="s">
-        <v>13</v>
+        <v>30</v>
       </c>
       <c r="J62" t="s">
-        <v>21</v>
+        <v>58</v>
       </c>
       <c r="L62">
         <v>4</v>
@@ -2789,17 +2793,17 @@
         <v>0</v>
       </c>
       <c r="O62">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>-8</v>
       </c>
       <c r="P62">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>8</v>
       </c>
     </row>
     <row r="64" spans="1:16" s="1" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A64" s="1" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B64" s="1" t="str">
         <f>A75</f>
@@ -2808,7 +2812,7 @@
     </row>
     <row r="65" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A65" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B65" t="str">
         <f>K75</f>
@@ -2817,7 +2821,7 @@
     </row>
     <row r="66" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A66" t="s">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="B66" t="str">
         <f>G75</f>
@@ -2826,7 +2830,7 @@
     </row>
     <row r="67" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A67" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B67" t="str">
         <f>I75</f>
@@ -2835,7 +2839,7 @@
     </row>
     <row r="68" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A68" t="s">
-        <v>91</v>
+        <v>6</v>
       </c>
       <c r="B68">
         <v>150000</v>
@@ -2843,7 +2847,7 @@
     </row>
     <row r="69" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A69" t="s">
-        <v>92</v>
+        <v>8</v>
       </c>
       <c r="B69">
         <v>16</v>
@@ -2851,7 +2855,7 @@
     </row>
     <row r="70" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A70" t="s">
-        <v>112</v>
+        <v>100</v>
       </c>
       <c r="B70">
         <v>20</v>
@@ -2859,7 +2863,7 @@
     </row>
     <row r="71" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A71" t="s">
-        <v>93</v>
+        <v>9</v>
       </c>
       <c r="B71">
         <v>8</v>
@@ -2867,23 +2871,23 @@
     </row>
     <row r="72" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A72" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="B72" t="s">
-        <v>102</v>
+        <v>11</v>
       </c>
     </row>
     <row r="73" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A73" s="1" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
     </row>
     <row r="74" spans="1:17" s="1" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A74" s="1" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="B74" s="1" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="C74" s="1">
         <v>2020</v>
@@ -2898,64 +2902,66 @@
         <v>2080</v>
       </c>
       <c r="G74" s="1" t="s">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H74" s="1" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="I74" s="1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J74" s="1" t="s">
-        <v>5</v>
+        <v>16</v>
       </c>
       <c r="K74" s="1" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L74" s="1" t="s">
-        <v>85</v>
+        <v>17</v>
       </c>
       <c r="M74" s="1" t="s">
-        <v>86</v>
+        <v>18</v>
       </c>
       <c r="N74" s="1" t="s">
-        <v>87</v>
+        <v>19</v>
       </c>
       <c r="O74" s="1" t="s">
-        <v>88</v>
+        <v>20</v>
       </c>
       <c r="P74" s="1" t="s">
-        <v>89</v>
+        <v>21</v>
       </c>
       <c r="Q74" s="1" t="s">
-        <v>90</v>
+        <v>22</v>
       </c>
     </row>
     <row r="75" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A75" t="s">
-        <v>83</v>
+        <v>101</v>
       </c>
       <c r="B75">
-        <v>1</v>
+        <f>B68</f>
+        <v>150000</v>
       </c>
       <c r="G75" t="s">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="I75" t="s">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="J75" t="s">
-        <v>12</v>
+        <v>26</v>
       </c>
       <c r="K75" t="s">
-        <v>84</v>
+        <v>27</v>
       </c>
     </row>
     <row r="76" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A76" t="s">
-        <v>75</v>
+        <v>102</v>
       </c>
       <c r="B76" s="2">
+        <f>-393</f>
         <v>-393</v>
       </c>
       <c r="C76" s="2"/>
@@ -2963,38 +2969,31 @@
       <c r="E76" s="2"/>
       <c r="F76" s="2"/>
       <c r="G76" t="s">
-        <v>3</v>
+        <v>29</v>
       </c>
       <c r="I76" t="s">
-        <v>13</v>
+        <v>30</v>
       </c>
       <c r="J76" t="s">
-        <v>14</v>
+        <v>31</v>
       </c>
       <c r="K76" t="s">
-        <v>76</v>
+        <v>103</v>
       </c>
       <c r="L76">
-        <v>2</v>
-      </c>
-      <c r="M76">
-        <v>10</v>
-      </c>
-      <c r="N76">
-        <v>0.3</v>
-      </c>
-      <c r="O76">
         <v>1</v>
       </c>
-      <c r="P76">
-        <v>16</v>
-      </c>
+      <c r="M76" s="7">
+        <v>17</v>
+      </c>
+      <c r="N76" s="7"/>
     </row>
     <row r="77" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A77" t="s">
-        <v>49</v>
+        <v>28</v>
       </c>
       <c r="B77" s="2">
+        <f>-0.15755937</f>
         <v>-0.15755937</v>
       </c>
       <c r="C77" s="2"/>
@@ -3002,37 +3001,33 @@
       <c r="E77" s="2"/>
       <c r="F77" s="2"/>
       <c r="G77" t="s">
-        <v>3</v>
+        <v>29</v>
       </c>
       <c r="I77" t="s">
-        <v>13</v>
+        <v>30</v>
       </c>
       <c r="J77" t="s">
-        <v>14</v>
+        <v>31</v>
       </c>
       <c r="K77" t="s">
-        <v>50</v>
+        <v>32</v>
       </c>
       <c r="L77">
         <v>4</v>
       </c>
-      <c r="M77">
-        <v>0</v>
-      </c>
       <c r="O77">
-        <f>$B$10-$B$9</f>
-        <v>-8</v>
+        <v>0</v>
       </c>
       <c r="P77">
-        <f>$B$9-$B$10</f>
-        <v>8</v>
+        <v>16</v>
       </c>
     </row>
     <row r="78" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A78" t="s">
-        <v>55</v>
+        <v>34</v>
       </c>
       <c r="B78" s="2">
+        <f>-1.73315307</f>
         <v>-1.73315307</v>
       </c>
       <c r="C78" s="2"/>
@@ -3040,111 +3035,98 @@
       <c r="E78" s="2"/>
       <c r="F78" s="2"/>
       <c r="G78" t="s">
-        <v>3</v>
+        <v>29</v>
       </c>
       <c r="I78" t="s">
-        <v>13</v>
+        <v>30</v>
       </c>
       <c r="J78" t="s">
-        <v>14</v>
+        <v>31</v>
       </c>
       <c r="K78" t="s">
-        <v>56</v>
+        <v>35</v>
       </c>
       <c r="L78">
         <v>4</v>
       </c>
-      <c r="M78">
-        <v>0</v>
-      </c>
       <c r="O78">
-        <f>$B$10-$B$9</f>
-        <v>-8</v>
+        <v>0</v>
       </c>
       <c r="P78">
-        <f>$B$9-$B$10</f>
-        <v>8</v>
+        <v>16</v>
       </c>
     </row>
     <row r="79" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A79" t="s">
-        <v>57</v>
+        <v>36</v>
       </c>
       <c r="B79" s="2">
-        <v>-10.135139250000002</v>
+        <f>-10.13513925</f>
+        <v>-10.13513925</v>
       </c>
       <c r="C79" s="2"/>
       <c r="D79" s="2"/>
       <c r="E79" s="2"/>
       <c r="F79" s="2"/>
       <c r="G79" t="s">
-        <v>3</v>
+        <v>29</v>
       </c>
       <c r="I79" t="s">
-        <v>13</v>
+        <v>30</v>
       </c>
       <c r="J79" t="s">
-        <v>14</v>
+        <v>31</v>
       </c>
       <c r="K79" t="s">
-        <v>58</v>
+        <v>37</v>
       </c>
       <c r="L79">
         <v>4</v>
       </c>
-      <c r="M79">
-        <v>0</v>
-      </c>
       <c r="O79">
-        <f>$B$10-$B$9</f>
-        <v>-8</v>
+        <v>0</v>
       </c>
       <c r="P79">
-        <f>$B$9-$B$10</f>
-        <v>8</v>
+        <v>16</v>
       </c>
     </row>
     <row r="80" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A80" t="s">
-        <v>77</v>
+        <v>104</v>
       </c>
       <c r="B80" s="2">
-        <v>1.0000000000000004</v>
+        <f>1</f>
+        <v>1</v>
       </c>
       <c r="C80" s="2"/>
       <c r="D80" s="2"/>
       <c r="E80" s="2"/>
       <c r="F80" s="2"/>
       <c r="G80" t="s">
-        <v>3</v>
+        <v>29</v>
       </c>
       <c r="I80" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J80" t="s">
-        <v>14</v>
+        <v>31</v>
       </c>
       <c r="K80" t="s">
-        <v>78</v>
+        <v>104</v>
       </c>
       <c r="L80">
         <v>4</v>
       </c>
-      <c r="M80">
-        <v>0</v>
-      </c>
       <c r="O80">
-        <f>$B$10-$B$9</f>
-        <v>-8</v>
+        <v>0</v>
       </c>
       <c r="P80">
-        <f>$B$9-$B$10</f>
-        <v>8</v>
+        <v>16</v>
       </c>
     </row>
     <row r="81" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A81" t="s">
-        <v>17</v>
+        <v>105</v>
       </c>
       <c r="B81" s="3">
         <f>B70/100*B68</f>
@@ -3155,37 +3137,33 @@
       <c r="E81" s="2"/>
       <c r="F81" s="2"/>
       <c r="G81" t="s">
+        <v>24</v>
+      </c>
+      <c r="I81" t="s">
+        <v>106</v>
+      </c>
+      <c r="J81" t="s">
+        <v>31</v>
+      </c>
+      <c r="K81" t="s">
+        <v>107</v>
+      </c>
+      <c r="L81">
+        <v>4</v>
+      </c>
+      <c r="O81">
+        <v>0</v>
+      </c>
+      <c r="P81">
         <v>16</v>
-      </c>
-      <c r="I81" t="s">
-        <v>18</v>
-      </c>
-      <c r="J81" t="s">
-        <v>14</v>
-      </c>
-      <c r="K81" t="s">
-        <v>19</v>
-      </c>
-      <c r="L81">
-        <v>4</v>
-      </c>
-      <c r="M81">
-        <v>0</v>
-      </c>
-      <c r="O81">
-        <f>$B$10-$B$9</f>
-        <v>-8</v>
-      </c>
-      <c r="P81">
-        <f>$B$9-$B$10</f>
-        <v>8</v>
       </c>
     </row>
     <row r="82" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A82" t="s">
-        <v>96</v>
+        <v>38</v>
       </c>
       <c r="B82" s="2">
+        <f>73.122</f>
         <v>73.122</v>
       </c>
       <c r="C82" s="2"/>
@@ -3193,22 +3171,19 @@
       <c r="E82" s="2"/>
       <c r="F82" s="2"/>
       <c r="G82" t="s">
-        <v>15</v>
+        <v>39</v>
       </c>
       <c r="I82" t="s">
-        <v>51</v>
+        <v>40</v>
       </c>
       <c r="J82" t="s">
-        <v>14</v>
+        <v>31</v>
       </c>
       <c r="K82" t="s">
-        <v>52</v>
+        <v>41</v>
       </c>
       <c r="L82">
         <v>4</v>
-      </c>
-      <c r="M82">
-        <v>-20</v>
       </c>
       <c r="O82">
         <v>-40</v>
@@ -3219,83 +3194,106 @@
     </row>
     <row r="83" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A83" t="s">
-        <v>95</v>
+        <v>47</v>
       </c>
       <c r="B83" s="2">
-        <v>918.22000000000048</v>
+        <v>39.799999999999997</v>
       </c>
       <c r="C83" s="2"/>
       <c r="D83" s="2"/>
       <c r="E83" s="2"/>
       <c r="F83" s="2"/>
       <c r="G83" t="s">
-        <v>3</v>
+        <v>50</v>
       </c>
       <c r="I83" t="s">
-        <v>13</v>
+        <v>40</v>
       </c>
       <c r="J83" t="s">
-        <v>14</v>
+        <v>31</v>
       </c>
       <c r="K83" t="s">
-        <v>79</v>
+        <v>47</v>
       </c>
       <c r="L83">
-        <v>2</v>
-      </c>
-      <c r="M83">
-        <f>-1*$B$71</f>
-        <v>-8</v>
-      </c>
-      <c r="N83">
-        <v>0.1</v>
+        <v>4</v>
       </c>
       <c r="O83">
-        <f>-1*B69</f>
-        <v>-16</v>
+        <v>0</v>
       </c>
       <c r="P83">
-        <v>-1</v>
+        <v>16</v>
       </c>
     </row>
     <row r="84" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A84" t="s">
-        <v>80</v>
+        <v>108</v>
       </c>
       <c r="B84" s="2">
-        <v>460</v>
+        <f>918.22</f>
+        <v>918.22</v>
       </c>
       <c r="C84" s="2"/>
       <c r="D84" s="2"/>
       <c r="E84" s="2"/>
       <c r="F84" s="2"/>
       <c r="G84" t="s">
-        <v>3</v>
+        <v>29</v>
       </c>
       <c r="I84" t="s">
-        <v>13</v>
+        <v>30</v>
       </c>
       <c r="J84" t="s">
-        <v>14</v>
+        <v>31</v>
       </c>
       <c r="K84" t="s">
-        <v>81</v>
+        <v>109</v>
       </c>
       <c r="L84">
-        <v>2</v>
-      </c>
-      <c r="M84">
-        <f>-1*$B$71</f>
-        <v>-8</v>
-      </c>
-      <c r="N84">
-        <v>0.1</v>
-      </c>
+        <v>4</v>
+      </c>
+      <c r="M84" s="7"/>
+      <c r="N84" s="7"/>
       <c r="O84">
-        <f>-1*B69</f>
-        <v>-16</v>
+        <v>-4</v>
       </c>
       <c r="P84">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="85" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A85" t="s">
+        <v>110</v>
+      </c>
+      <c r="B85" s="2">
+        <f>460</f>
+        <v>460</v>
+      </c>
+      <c r="C85" s="2"/>
+      <c r="D85" s="2"/>
+      <c r="E85" s="2"/>
+      <c r="F85" s="2"/>
+      <c r="G85" t="s">
+        <v>111</v>
+      </c>
+      <c r="I85" t="s">
+        <v>30</v>
+      </c>
+      <c r="J85" t="s">
+        <v>31</v>
+      </c>
+      <c r="K85" t="s">
+        <v>112</v>
+      </c>
+      <c r="L85">
+        <v>4</v>
+      </c>
+      <c r="M85" s="7"/>
+      <c r="N85" s="7"/>
+      <c r="O85">
+        <v>-3</v>
+      </c>
+      <c r="P85">
         <v>-1</v>
       </c>
     </row>
@@ -3305,7 +3303,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4EB8EA02-EB39-D140-B9BA-474DA0F5EB60}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:T35"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
@@ -3317,7 +3315,7 @@
   <sheetData>
     <row r="1" spans="1:18" s="1" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B1" s="1" t="str">
         <f>A13</f>
@@ -3326,15 +3324,15 @@
     </row>
     <row r="2" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B2" t="s">
-        <v>128</v>
+        <v>113</v>
       </c>
     </row>
     <row r="3" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="B3" t="str">
         <f>G13</f>
@@ -3343,7 +3341,7 @@
     </row>
     <row r="4" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B4" t="str">
         <f>I13</f>
@@ -3352,7 +3350,7 @@
     </row>
     <row r="5" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>126</v>
+        <v>114</v>
       </c>
       <c r="B5">
         <v>30</v>
@@ -3360,7 +3358,7 @@
     </row>
     <row r="6" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>122</v>
+        <v>115</v>
       </c>
       <c r="B6">
         <v>20</v>
@@ -3368,7 +3366,7 @@
     </row>
     <row r="7" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>123</v>
+        <v>116</v>
       </c>
       <c r="B7">
         <v>0.81</v>
@@ -3376,7 +3374,7 @@
     </row>
     <row r="8" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>124</v>
+        <v>117</v>
       </c>
       <c r="B8">
         <v>1600</v>
@@ -3384,7 +3382,7 @@
     </row>
     <row r="9" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>125</v>
+        <v>118</v>
       </c>
       <c r="B9" s="5">
         <f>B8*B5*3.6</f>
@@ -3393,23 +3391,23 @@
     </row>
     <row r="10" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="B10" t="s">
-        <v>102</v>
+        <v>11</v>
       </c>
     </row>
     <row r="11" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A11" s="1" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
     </row>
     <row r="12" spans="1:18" s="1" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A12" s="1" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="C12" s="1">
         <v>2020</v>
@@ -3424,81 +3422,81 @@
         <v>2080</v>
       </c>
       <c r="G12" s="1" t="s">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H12" s="1" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="I12" s="1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J12" s="1" t="s">
-        <v>5</v>
+        <v>16</v>
       </c>
       <c r="K12" s="1" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L12" s="1" t="s">
-        <v>85</v>
+        <v>17</v>
       </c>
       <c r="M12" s="1" t="s">
-        <v>86</v>
+        <v>18</v>
       </c>
       <c r="N12" s="1" t="s">
-        <v>87</v>
+        <v>19</v>
       </c>
       <c r="O12" s="1" t="s">
-        <v>88</v>
+        <v>20</v>
       </c>
       <c r="P12" s="1" t="s">
-        <v>89</v>
+        <v>21</v>
       </c>
       <c r="Q12" s="1" t="s">
-        <v>90</v>
+        <v>22</v>
       </c>
       <c r="R12" s="1" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
     </row>
     <row r="13" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
       <c r="B13" s="6">
         <f>B9</f>
         <v>172800</v>
       </c>
       <c r="G13" t="s">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="I13" t="s">
-        <v>127</v>
+        <v>120</v>
       </c>
       <c r="J13" t="s">
-        <v>12</v>
+        <v>26</v>
       </c>
       <c r="K13" t="s">
-        <v>128</v>
+        <v>113</v>
       </c>
     </row>
     <row r="14" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>115</v>
+        <v>121</v>
       </c>
       <c r="B14">
-        <v>13305.600000000017</v>
+        <v>13305.60000000002</v>
       </c>
       <c r="G14" t="s">
-        <v>117</v>
+        <v>122</v>
       </c>
       <c r="I14" t="s">
-        <v>13</v>
+        <v>30</v>
       </c>
       <c r="J14" t="s">
-        <v>14</v>
+        <v>31</v>
       </c>
       <c r="K14" t="s">
-        <v>116</v>
+        <v>123</v>
       </c>
       <c r="L14">
         <v>4</v>
@@ -3512,22 +3510,22 @@
     </row>
     <row r="15" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>114</v>
+        <v>124</v>
       </c>
       <c r="B15" s="4">
         <v>5.3333333333333337E-2</v>
       </c>
       <c r="G15" t="s">
-        <v>117</v>
+        <v>122</v>
       </c>
       <c r="I15" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J15" t="s">
-        <v>14</v>
+        <v>31</v>
       </c>
       <c r="K15" t="s">
-        <v>118</v>
+        <v>125</v>
       </c>
       <c r="L15">
         <v>3</v>
@@ -3547,22 +3545,22 @@
     </row>
     <row r="16" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>119</v>
+        <v>126</v>
       </c>
       <c r="B16">
         <v>686.26285714285859</v>
       </c>
       <c r="G16" t="s">
-        <v>117</v>
+        <v>122</v>
       </c>
       <c r="I16" t="s">
-        <v>18</v>
+        <v>106</v>
       </c>
       <c r="J16" t="s">
-        <v>14</v>
+        <v>31</v>
       </c>
       <c r="K16" t="s">
-        <v>19</v>
+        <v>107</v>
       </c>
       <c r="L16">
         <v>4</v>
@@ -3576,19 +3574,19 @@
     </row>
     <row r="17" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>103</v>
+        <v>59</v>
       </c>
       <c r="B17">
-        <v>24216.685714285693</v>
+        <v>24216.68571428569</v>
       </c>
       <c r="H17" t="s">
-        <v>22</v>
+        <v>57</v>
       </c>
       <c r="I17" t="s">
-        <v>13</v>
+        <v>30</v>
       </c>
       <c r="J17" t="s">
-        <v>21</v>
+        <v>58</v>
       </c>
       <c r="L17">
         <v>4</v>
@@ -3602,22 +3600,22 @@
     </row>
     <row r="18" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B18">
         <v>-96.767999999999986</v>
       </c>
       <c r="G18" t="s">
-        <v>117</v>
+        <v>122</v>
       </c>
       <c r="I18" t="s">
-        <v>13</v>
+        <v>30</v>
       </c>
       <c r="J18" t="s">
-        <v>14</v>
+        <v>31</v>
       </c>
       <c r="K18" t="s">
-        <v>121</v>
+        <v>128</v>
       </c>
       <c r="L18">
         <v>4</v>
@@ -3631,7 +3629,7 @@
     </row>
     <row r="20" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A20" s="1" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B20" s="1" t="str">
         <f>A32</f>
@@ -3640,15 +3638,15 @@
     </row>
     <row r="21" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B21" t="s">
-        <v>128</v>
+        <v>113</v>
       </c>
     </row>
     <row r="22" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="B22" t="str">
         <f>G32</f>
@@ -3657,7 +3655,7 @@
     </row>
     <row r="23" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B23" t="str">
         <f>I32</f>
@@ -3666,7 +3664,7 @@
     </row>
     <row r="24" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>126</v>
+        <v>114</v>
       </c>
       <c r="B24">
         <v>30</v>
@@ -3674,7 +3672,7 @@
     </row>
     <row r="25" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>122</v>
+        <v>115</v>
       </c>
       <c r="B25">
         <v>20</v>
@@ -3682,7 +3680,7 @@
     </row>
     <row r="26" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>123</v>
+        <v>116</v>
       </c>
       <c r="B26">
         <v>2.8</v>
@@ -3690,7 +3688,7 @@
     </row>
     <row r="27" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>124</v>
+        <v>117</v>
       </c>
       <c r="B27">
         <v>1600</v>
@@ -3698,7 +3696,7 @@
     </row>
     <row r="28" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>125</v>
+        <v>118</v>
       </c>
       <c r="B28" s="5">
         <f>B27*B24*3.6</f>
@@ -3707,23 +3705,23 @@
     </row>
     <row r="29" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="B29" t="s">
-        <v>102</v>
+        <v>11</v>
       </c>
     </row>
     <row r="30" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A30" s="1" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
     </row>
     <row r="31" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A31" s="1" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="C31" s="1">
         <v>2020</v>
@@ -3738,94 +3736,94 @@
         <v>2080</v>
       </c>
       <c r="G31" s="1" t="s">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H31" s="1" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="I31" s="1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J31" s="1" t="s">
-        <v>5</v>
+        <v>16</v>
       </c>
       <c r="K31" s="1" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L31" s="1" t="s">
-        <v>85</v>
+        <v>17</v>
       </c>
       <c r="M31" s="1" t="s">
-        <v>86</v>
+        <v>18</v>
       </c>
       <c r="N31" s="1" t="s">
-        <v>87</v>
+        <v>19</v>
       </c>
       <c r="O31" s="1" t="s">
-        <v>88</v>
+        <v>20</v>
       </c>
       <c r="P31" s="1" t="s">
-        <v>89</v>
+        <v>21</v>
       </c>
       <c r="Q31" s="1" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="R31" s="1" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="S31" s="1" t="s">
-        <v>90</v>
+        <v>22</v>
       </c>
       <c r="T31" s="1" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
     </row>
     <row r="32" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="B32" s="6">
         <f>B28</f>
         <v>172800</v>
       </c>
       <c r="G32" t="s">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="I32" t="s">
-        <v>127</v>
+        <v>120</v>
       </c>
       <c r="J32" t="s">
-        <v>12</v>
+        <v>26</v>
       </c>
       <c r="K32" t="s">
-        <v>128</v>
+        <v>113</v>
       </c>
     </row>
     <row r="33" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="B33" s="4">
         <f>0.00599616*2</f>
         <v>1.1992320000000001E-2</v>
       </c>
       <c r="G33" t="s">
-        <v>3</v>
+        <v>29</v>
       </c>
       <c r="I33" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J33" t="s">
-        <v>14</v>
+        <v>31</v>
       </c>
       <c r="K33" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="L33">
         <v>6</v>
       </c>
       <c r="Q33" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="R33" t="s">
         <v>135</v>
@@ -3833,23 +3831,23 @@
     </row>
     <row r="34" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
-        <v>17</v>
+        <v>105</v>
       </c>
       <c r="B34" s="6">
         <f>B32/2.9/3.6</f>
         <v>16551.724137931033</v>
       </c>
       <c r="G34" t="s">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="I34" t="s">
-        <v>18</v>
+        <v>106</v>
       </c>
       <c r="J34" t="s">
-        <v>14</v>
+        <v>31</v>
       </c>
       <c r="K34" t="s">
-        <v>19</v>
+        <v>107</v>
       </c>
       <c r="L34">
         <v>4</v>
@@ -3863,19 +3861,19 @@
     </row>
     <row r="35" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
-        <v>132</v>
+        <v>136</v>
       </c>
       <c r="B35" s="4">
         <v>6.7910399999999996E-2</v>
       </c>
       <c r="H35" t="s">
-        <v>22</v>
+        <v>57</v>
       </c>
       <c r="I35" t="s">
-        <v>13</v>
+        <v>30</v>
       </c>
       <c r="J35" t="s">
-        <v>21</v>
+        <v>58</v>
       </c>
       <c r="L35">
         <v>4</v>

</xml_diff>